<commit_message>
finally added the carmodule and google login module MODIFIED
</commit_message>
<xml_diff>
--- a/src/test/resources/Details.xlsx
+++ b/src/test/resources/Details.xlsx
@@ -3,21 +3,22 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2497760\Ideaprojects\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F12C0AC9-9A3D-49DB-9861-5AE55ECAA867}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{412D0D53-2C7B-444A-A8FB-D529F36BD621}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{BAA70594-9921-46EE-9B36-55EF6409868E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="CarDetails" r:id="rId5" sheetId="2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -38,8 +39,74 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="20">
+  <si>
+    <t>Honda City 1.5 S MT</t>
+  </si>
+  <si>
+    <t>Rs. 4.60 Lakh</t>
+  </si>
+  <si>
+    <t>Honda City 1.5 V MT Exclusive</t>
+  </si>
+  <si>
+    <t>Rs. 4.55 Lakh</t>
+  </si>
+  <si>
+    <t>Hyundai i10 Magna</t>
+  </si>
+  <si>
+    <t>Rs. 3.20 Lakh</t>
+  </si>
+  <si>
+    <t>Honda City SV MT</t>
+  </si>
+  <si>
+    <t>Rs. 5.15 Lakh</t>
+  </si>
+  <si>
+    <t>Hyundai i10 Sportz 1.1L</t>
+  </si>
+  <si>
+    <t>Rs. 3.65 Lakh</t>
+  </si>
+  <si>
+    <t>Rs. 4.70 Lakh</t>
+  </si>
+  <si>
+    <t>Rs. 3.25 Lakh</t>
+  </si>
+  <si>
+    <t>Honda City i VTEC CVT VX</t>
+  </si>
+  <si>
+    <t>Rs. 4.84 Lakh</t>
+  </si>
+  <si>
+    <t>Honda City V MT</t>
+  </si>
+  <si>
+    <t>Rs. 6.70 Lakh</t>
+  </si>
+  <si>
+    <t>Honda City ZX MT</t>
+  </si>
+  <si>
+    <t>Rs. 9.25 Lakh</t>
+  </si>
+  <si>
+    <t>Honda City i VTEC V</t>
+  </si>
+  <si>
+    <t>Rs. 6.90 Lakh</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="0"/>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -410,4 +477,102 @@
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:B11"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="B8" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="B9" t="s" s="0">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="B10" t="s" s="0">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="B11" t="s" s="0">
+        <v>19</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Merged all the testcases
</commit_message>
<xml_diff>
--- a/src/test/resources/Details.xlsx
+++ b/src/test/resources/Details.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2497760\Ideaprojects\src\test\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2497739\IdeaProjects\IdentifyNewBikes\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E008CE4-57D5-4C0C-A354-35351A46C240}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78C17B0B-E170-4C7E-B2E9-7C9BF4EAF7A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{BAA70594-9921-46EE-9B36-55EF6409868E}"/>
   </bookViews>

</xml_diff>